<commit_message>
New changes in custom agents
</commit_message>
<xml_diff>
--- a/Ui Automation Test Report.xlsx
+++ b/Ui Automation Test Report.xlsx
@@ -5561,7 +5561,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:G8"/>
+  <dimension ref="A1:G20"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" style="23" min="1" max="1"/>
@@ -5682,30 +5682,94 @@
     <row r="5">
       <c r="A5" s="26" t="inlineStr">
         <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="B5" s="27" t="n">
+        <v>13</v>
+      </c>
+      <c r="C5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F5" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G5" s="27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="6">
+      <c r="A6" s="26" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="B6" s="27" t="n">
+        <v>19</v>
+      </c>
+      <c r="C6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="D6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="E6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="F6" s="27" t="n">
+        <v>0</v>
+      </c>
+      <c r="G6" s="27" t="n">
+        <v>0</v>
+      </c>
+    </row>
+    <row r="7">
+      <c r="A7" s="26" t="inlineStr">
+        <is>
           <t>Total</t>
         </is>
       </c>
-      <c r="B5" s="27" t="n">
-        <v>17</v>
-      </c>
-    </row>
-    <row r="7">
-      <c r="A7" s="28" t="inlineStr">
+      <c r="B7" s="27" t="n">
+        <v>49</v>
+      </c>
+    </row>
+    <row r="8">
+      <c r="A8" s="28" t="n"/>
+      <c r="B8" s="29" t="n"/>
+    </row>
+    <row r="9">
+      <c r="A9" s="28" t="inlineStr">
         <is>
           <t>Milestone Dates</t>
         </is>
       </c>
     </row>
-    <row r="8">
-      <c r="A8" s="28" t="inlineStr">
+    <row r="10">
+      <c r="A10" s="28" t="inlineStr">
         <is>
           <t xml:space="preserve"> july1st </t>
         </is>
       </c>
-      <c r="B8" s="29" t="n">
+      <c r="B10" s="29" t="n">
         <v>46216</v>
       </c>
     </row>
+    <row r="11"/>
+    <row r="12"/>
+    <row r="13"/>
+    <row r="14"/>
+    <row r="15"/>
+    <row r="16"/>
+    <row r="17"/>
+    <row r="18"/>
+    <row r="19"/>
+    <row r="20"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5717,7 +5781,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:H18"/>
+  <dimension ref="A1:H50"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="19.88" customWidth="1" style="23" min="1" max="1"/>
@@ -6311,6 +6375,1030 @@
         </is>
       </c>
     </row>
+    <row r="19">
+      <c r="A19" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B19" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C19" s="31" t="inlineStr">
+        <is>
+          <t>BJ01</t>
+        </is>
+      </c>
+      <c r="D19" s="31" t="inlineStr">
+        <is>
+          <t>POST preview cron (cron_expression, timezone) — verify 200, valid=true, error null, next_runs is a non-empty list of 5</t>
+        </is>
+      </c>
+      <c r="E19" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F19" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="20">
+      <c r="A20" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B20" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C20" s="31" t="inlineStr">
+        <is>
+          <t>BJ02</t>
+        </is>
+      </c>
+      <c r="D20" s="31" t="inlineStr">
+        <is>
+          <t>GET can-create background job — verify 200, canCreateBackgroundJob present as a bool matching the role</t>
+        </is>
+      </c>
+      <c r="E20" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F20" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="21">
+      <c r="A21" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B21" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C21" s="31" t="inlineStr">
+        <is>
+          <t>BJ03</t>
+        </is>
+      </c>
+      <c r="D21" s="31" t="inlineStr">
+        <is>
+          <t>POST create background job (project_id, agent, cron, name) — verify 201, job_id returned, status=active, trigger_type=scheduled</t>
+        </is>
+      </c>
+      <c r="E21" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F21" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="22">
+      <c r="A22" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B22" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C22" s="31" t="inlineStr">
+        <is>
+          <t>BJ04</t>
+        </is>
+      </c>
+      <c r="D22" s="31" t="inlineStr">
+        <is>
+          <t>GET list background jobs (project_id, mine_only, include_removed) — verify 200, jobs+total, schema keys, all scoped to project</t>
+        </is>
+      </c>
+      <c r="E22" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F22" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="23">
+      <c r="A23" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B23" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C23" s="31" t="inlineStr">
+        <is>
+          <t>BJ05</t>
+        </is>
+      </c>
+      <c r="D23" s="31" t="inlineStr">
+        <is>
+          <t>GET admin list all background jobs (include_removed) — verify 200, jobs+total, schema keys incl. project_name</t>
+        </is>
+      </c>
+      <c r="E23" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F23" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="24">
+      <c r="A24" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B24" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C24" s="31" t="inlineStr">
+        <is>
+          <t>BJ06</t>
+        </is>
+      </c>
+      <c r="D24" s="31" t="inlineStr">
+        <is>
+          <t>PATCH update background job (name/prompt/cron) — verify 200, job_id unchanged, edited fields echoed with new values</t>
+        </is>
+      </c>
+      <c r="E24" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F24" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="25">
+      <c r="A25" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B25" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C25" s="31" t="inlineStr">
+        <is>
+          <t>BJ07</t>
+        </is>
+      </c>
+      <c r="D25" s="31" t="inlineStr">
+        <is>
+          <t>GET background job — verify 200, returned job_id matches, payload carries expected schema keys</t>
+        </is>
+      </c>
+      <c r="E25" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F25" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="26">
+      <c r="A26" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B26" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C26" s="31" t="inlineStr">
+        <is>
+          <t>BJ08</t>
+        </is>
+      </c>
+      <c r="D26" s="31" t="inlineStr">
+        <is>
+          <t>POST run background job now — verify 200, job_id matches, status=queued, task_id returned</t>
+        </is>
+      </c>
+      <c r="E26" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F26" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="27">
+      <c r="A27" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B27" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C27" s="31" t="inlineStr">
+        <is>
+          <t>BJ09</t>
+        </is>
+      </c>
+      <c r="D27" s="31" t="inlineStr">
+        <is>
+          <t>POST pause background job — verify 200, job_id matches, status=paused, next_run_at null</t>
+        </is>
+      </c>
+      <c r="E27" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F27" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="28">
+      <c r="A28" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B28" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C28" s="31" t="inlineStr">
+        <is>
+          <t>BJ10</t>
+        </is>
+      </c>
+      <c r="D28" s="31" t="inlineStr">
+        <is>
+          <t>POST resume background job — verify 200, job_id matches, status=active, next_run_at re-registered</t>
+        </is>
+      </c>
+      <c r="E28" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F28" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="29">
+      <c r="A29" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B29" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C29" s="31" t="inlineStr">
+        <is>
+          <t>BJ11</t>
+        </is>
+      </c>
+      <c r="D29" s="31" t="inlineStr">
+        <is>
+          <t>GET background job runs — verify 200, runs list + aggregates, succeeded+failed==total_runs, success_rate in [0,1]</t>
+        </is>
+      </c>
+      <c r="E29" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F29" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="30">
+      <c r="A30" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B30" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C30" s="31" t="inlineStr">
+        <is>
+          <t>BJ12</t>
+        </is>
+      </c>
+      <c r="D30" s="31" t="inlineStr">
+        <is>
+          <t>GET background job run detail — verify 200, job_id+message_id match, output present, timeline list, usage keys</t>
+        </is>
+      </c>
+      <c r="E30" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F30" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="31">
+      <c r="A31" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B31" s="31" t="inlineStr">
+        <is>
+          <t>Background Jobs</t>
+        </is>
+      </c>
+      <c r="C31" s="31" t="inlineStr">
+        <is>
+          <t>BJ13</t>
+        </is>
+      </c>
+      <c r="D31" s="31" t="inlineStr">
+        <is>
+          <t>DELETE remove background job — verify 200, job_id matches, status=removed, next_run_at null</t>
+        </is>
+      </c>
+      <c r="E31" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F31" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="32">
+      <c r="A32" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B32" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C32" s="31" t="inlineStr">
+        <is>
+          <t>CA01</t>
+        </is>
+      </c>
+      <c r="D32" s="31" t="inlineStr">
+        <is>
+          <t>POST onboard custom agent from .ncp package — verify 200, success message, agent_id, agent_name, status=ACTIVE</t>
+        </is>
+      </c>
+      <c r="E32" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F32" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="33">
+      <c r="A33" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B33" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C33" s="31" t="inlineStr">
+        <is>
+          <t>CA02</t>
+        </is>
+      </c>
+      <c r="D33" s="31" t="inlineStr">
+        <is>
+          <t>GET list custom agents — verify 200, agents+total present, total matches count, schema keys present</t>
+        </is>
+      </c>
+      <c r="E33" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F33" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="34">
+      <c r="A34" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B34" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C34" s="31" t="inlineStr">
+        <is>
+          <t>CA03</t>
+        </is>
+      </c>
+      <c r="D34" s="31" t="inlineStr">
+        <is>
+          <t>GET background-eligible custom agents — verify 200, agents+total, schema keys, every agent status=ACTIVE</t>
+        </is>
+      </c>
+      <c r="E34" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F34" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="35">
+      <c r="A35" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B35" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C35" s="31" t="inlineStr">
+        <is>
+          <t>CA04</t>
+        </is>
+      </c>
+      <c r="D35" s="31" t="inlineStr">
+        <is>
+          <t>GET custom agent by name — verify 200, returned name matches, payload carries schema keys</t>
+        </is>
+      </c>
+      <c r="E35" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F35" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="36">
+      <c r="A36" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B36" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C36" s="31" t="inlineStr">
+        <is>
+          <t>CA05</t>
+        </is>
+      </c>
+      <c r="D36" s="31" t="inlineStr">
+        <is>
+          <t>POST disable custom agent — verify 200, agent_name matches, status=DISABLED, message returned</t>
+        </is>
+      </c>
+      <c r="E36" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F36" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="37">
+      <c r="A37" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B37" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C37" s="31" t="inlineStr">
+        <is>
+          <t>CA06</t>
+        </is>
+      </c>
+      <c r="D37" s="31" t="inlineStr">
+        <is>
+          <t>POST enable custom agent — verify 200, agent_name matches, status=ACTIVE, message returned</t>
+        </is>
+      </c>
+      <c r="E37" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F37" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="38">
+      <c r="A38" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B38" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C38" s="31" t="inlineStr">
+        <is>
+          <t>CA07</t>
+        </is>
+      </c>
+      <c r="D38" s="31" t="inlineStr">
+        <is>
+          <t>POST enable-background custom agent — verify 200, agent_name matches, supports_background=true</t>
+        </is>
+      </c>
+      <c r="E38" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F38" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="39">
+      <c r="A39" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B39" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C39" s="31" t="inlineStr">
+        <is>
+          <t>CA08</t>
+        </is>
+      </c>
+      <c r="D39" s="31" t="inlineStr">
+        <is>
+          <t>POST disable-background custom agent — verify 200, agent_name matches, supports_background=false</t>
+        </is>
+      </c>
+      <c r="E39" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F39" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="40">
+      <c r="A40" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B40" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C40" s="31" t="inlineStr">
+        <is>
+          <t>CA09</t>
+        </is>
+      </c>
+      <c r="D40" s="31" t="inlineStr">
+        <is>
+          <t>GET admin list custom agents — verify 200, agents+total, admin schema keys incl. assigned_roles (a list)</t>
+        </is>
+      </c>
+      <c r="E40" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F40" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="41">
+      <c r="A41" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B41" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C41" s="31" t="inlineStr">
+        <is>
+          <t>CA10</t>
+        </is>
+      </c>
+      <c r="D41" s="31" t="inlineStr">
+        <is>
+          <t>GET my custom agents — verify 200, agents+total, schema keys, every agent submitted_by the caller</t>
+        </is>
+      </c>
+      <c r="E41" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F41" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="42">
+      <c r="A42" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B42" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C42" s="31" t="inlineStr">
+        <is>
+          <t>CA11</t>
+        </is>
+      </c>
+      <c r="D42" s="31" t="inlineStr">
+        <is>
+          <t>POST submit custom agent (.ncp) — verify 200, agent_id, agent_name, status ACTIVE (admin) or PENDING (user)</t>
+        </is>
+      </c>
+      <c r="E42" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F42" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="43">
+      <c r="A43" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B43" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C43" s="31" t="inlineStr">
+        <is>
+          <t>CA12</t>
+        </is>
+      </c>
+      <c r="D43" s="31" t="inlineStr">
+        <is>
+          <t>POST update custom agent new version (.ncp) — verify 200, agent_id matches, version returned, status ACTIVE/PENDING</t>
+        </is>
+      </c>
+      <c r="E43" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F43" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="44">
+      <c r="A44" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B44" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C44" s="31" t="inlineStr">
+        <is>
+          <t>CA13</t>
+        </is>
+      </c>
+      <c r="D44" s="31" t="inlineStr">
+        <is>
+          <t>POST approve custom agent — verify 200, agent_name matches, status=ACTIVE, message returned</t>
+        </is>
+      </c>
+      <c r="E44" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F44" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="45">
+      <c r="A45" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B45" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C45" s="31" t="inlineStr">
+        <is>
+          <t>CA14</t>
+        </is>
+      </c>
+      <c r="D45" s="31" t="inlineStr">
+        <is>
+          <t>POST decline custom agent (feedback) — verify 200, agent_name matches, status=REJECTED, message returned</t>
+        </is>
+      </c>
+      <c r="E45" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F45" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="46">
+      <c r="A46" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B46" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C46" s="31" t="inlineStr">
+        <is>
+          <t>CA15</t>
+        </is>
+      </c>
+      <c r="D46" s="31" t="inlineStr">
+        <is>
+          <t>POST feedback custom agent (message, feedback_type) — verify 200, agent_name matches, confirmation message</t>
+        </is>
+      </c>
+      <c r="E46" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F46" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B47" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C47" s="31" t="inlineStr">
+        <is>
+          <t>CA16</t>
+        </is>
+      </c>
+      <c r="D47" s="31" t="inlineStr">
+        <is>
+          <t>GET download custom agent package — verify 200, Content-Disposition .ncp attachment, non-empty bytes</t>
+        </is>
+      </c>
+      <c r="E47" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F47" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B48" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C48" s="31" t="inlineStr">
+        <is>
+          <t>CA17</t>
+        </is>
+      </c>
+      <c r="D48" s="31" t="inlineStr">
+        <is>
+          <t>GET can-submit-agent — verify 200, submitAgent present as a bool matching the role</t>
+        </is>
+      </c>
+      <c r="E48" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F48" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B49" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C49" s="31" t="inlineStr">
+        <is>
+          <t>CA18</t>
+        </is>
+      </c>
+      <c r="D49" s="31" t="inlineStr">
+        <is>
+          <t>DELETE remove custom agent (admin) — verify 200, agent_name matches, removal-confirmation message</t>
+        </is>
+      </c>
+      <c r="E49" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F49" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
+    <row r="50">
+      <c r="A50" s="31" t="inlineStr">
+        <is>
+          <t>Exposed API</t>
+        </is>
+      </c>
+      <c r="B50" s="31" t="inlineStr">
+        <is>
+          <t>Custom Agents</t>
+        </is>
+      </c>
+      <c r="C50" s="31" t="inlineStr">
+        <is>
+          <t>CA19</t>
+        </is>
+      </c>
+      <c r="D50" s="31" t="inlineStr">
+        <is>
+          <t>DELETE remove user custom agent (allow_force_delete) — verify 200, agent_name matches, removal-confirmation message</t>
+        </is>
+      </c>
+      <c r="E50" s="31" t="inlineStr">
+        <is>
+          <t>Medium</t>
+        </is>
+      </c>
+      <c r="F50" s="31" t="inlineStr">
+        <is>
+          <t>Not Run</t>
+        </is>
+      </c>
+    </row>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>